<commit_message>
20° Commit- aggiornamenti in data  26.02.2026
</commit_message>
<xml_diff>
--- a/activity_code/activity_Code_list_protocolCore.xlsx
+++ b/activity_code/activity_Code_list_protocolCore.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mcorbara\Documents\ArgoX3_API_Mobile_CORE\activity_code\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{616B14C4-9AAA-43D9-A6BC-386EE1AFE006}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38E86079-EB56-46F2-87DC-B68FB5A0644B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Elenco codici attività" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="9">
   <si>
     <t>Codice</t>
   </si>
@@ -52,9 +52,6 @@
   </si>
   <si>
     <t>Patch</t>
-  </si>
-  <si>
-    <t>manca</t>
   </si>
 </sst>
 </file>
@@ -146,7 +143,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -472,9 +469,6 @@
       <c r="C3" t="s">
         <v>3</v>
       </c>
-      <c r="D3" t="s">
-        <v>9</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>